<commit_message>
docs(task-13): align platform onboarding workbook
</commit_message>
<xml_diff>
--- a/docs/client-materials/IVYBM_海外平台账号申请资料收集表.xlsx
+++ b/docs/client-materials/IVYBM_海外平台账号申请资料收集表.xlsx
@@ -164,94 +164,165 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">文档版本：2026-07-25    最后更新：2026-07-25    适用范围：海外平台账号申请资料收集（客户侧、非密）</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">填写原则</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1. 没有现成账号时，请在对应工作表填写“需新建”及希望使用的账号名；技术团队代为开设与配置。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">2. 企业主体、品牌、页面和开发者应用最终归客户公司所有；请指定可接收验证码并完成最终接管的负责人。</t>
+          <t xml:space="preserve">1. 没有现成账号时，请在对应工作表填写“需新建”及希望使用的账号名；技术团队代为开设与配置。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">3. 营业执照、身份证明等高敏感资料请通过受控文件夹或客户指定邮箱提供，只在表中写文件名或交付状态。</t>
+          <t xml:space="preserve">2. 企业主体、品牌、页面和开发者应用最终归客户公司所有；请指定可接收验证码并完成最终接管的负责人。</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">3. 营业执照、身份证明等高敏感资料请通过受控文件夹或客户指定邮箱提供，只在表中写文件名或交付状态。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">4. 所有“必填”项会影响账号创建、App Review 或真实联调；“建议”项可后补，但会延长审核时间。</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">当前一期范围</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Meta：Facebook Messenger、Instagram DM 入站；Facebook / Instagram 图文发布。</t>
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5. 本表仅收集非密资料：外部账号 ID、授权状态、审批状态、部署确认等，绝对不要填密码、App Secret、Client Secret、OAuth Token、银行卡或验证码。</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LinkedIn：图文发布；LinkedIn 私信不属于一期自动接入范围。</t>
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当前一期范围（冻结）</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TikTok：私信能力需先确认目标地区及官方 Business Messaging API 资格，当前为条件阻塞。</t>
+          <t xml:space="preserve">入站：Meta Facebook Messenger、Instagram DM、TikTok DM（TikTok 官方私信 schema 与 API 资格当前阻塞 / 待确认，不承诺自动接入）。</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">WhatsApp：不属于一期系统接入范围，请勿为本期申请。</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+          <t xml:space="preserve">出站（图文发布）：Meta Facebook / Instagram（一期受 PublishJobs / PublishLogs / adapter 设计评审约束，暂不承诺自动联调）；LinkedIn 个人主页 / 企业主页（保留辅助导出 fallback）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">排除：WhatsApp 不进入一期系统接入；LinkedIn 私信不属于一期自动接入范围。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">字段口径说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Meta：区分 facebook-page 与 instagram-professional；分别填写外部 Page ID / Professional Account ID、授权状态、消息入站审批状态、图文发布审批状态，以及 allowlist / App Secret / Verify Token 部署确认（仅状态）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LinkedIn：区分 linkedin-member（个人管理员）与 linkedin-organization（企业主页）；分别填写目标外部 ID、授权状态、发布 API 审批状态，以及客户侧 Super Admin 指定。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TikTok：tiktok-business 填写外部账号 ID、授权状态；私信 schema 与 API 资格当前统一标记为“被阻塞 / 待官方确认”，订单前再次确认，不承诺自动接入。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通用：所有“状态”列只填枚举值；不要把实际 secret、token、私信 schema 原文粘贴进表。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">状态下拉说明</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">未开始：尚未准备；已提供：已通过受控方式交付；待补充：资料不完整；不适用：确认无需提供。</t>
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">授权状态枚举：未开始、待处理、已连接、已过期、被阻塞、已停用。</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">审批状态枚举：未开始、待审核、已通过、被阻塞。</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">部署确认枚举：待确认、已确认部署、无需部署、被阻塞。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TikTok 私信当前口径枚举：待官方确认、被阻塞、暂不可用。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:H3"/>
   </mergeCells>
 </worksheet>
 </file>
@@ -358,7 +429,7 @@
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H5" s="11" t="inlineStr">
@@ -400,7 +471,7 @@
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
@@ -442,7 +513,7 @@
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H7" s="11" t="inlineStr">
@@ -484,7 +555,7 @@
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
@@ -526,7 +597,7 @@
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H9" s="11" t="inlineStr">
@@ -568,7 +639,7 @@
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
@@ -610,7 +681,7 @@
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H11" s="11" t="inlineStr">
@@ -652,7 +723,7 @@
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
@@ -694,7 +765,7 @@
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H13" s="11" t="inlineStr">
@@ -736,7 +807,7 @@
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
@@ -778,7 +849,7 @@
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H15" s="11" t="inlineStr">
@@ -820,7 +891,7 @@
       </c>
       <c r="G16" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -945,7 +1016,7 @@
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H5" s="11" t="inlineStr">
@@ -987,7 +1058,7 @@
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
@@ -1029,7 +1100,7 @@
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H7" s="11" t="inlineStr">
@@ -1071,7 +1142,7 @@
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
@@ -1113,7 +1184,7 @@
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H9" s="11" t="inlineStr">
@@ -1155,7 +1226,7 @@
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
@@ -1197,7 +1268,7 @@
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H11" s="11" t="inlineStr">
@@ -1239,7 +1310,7 @@
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
@@ -1261,7 +1332,7 @@
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">预生产 / 联调子域名</t>
+          <t xml:space="preserve">生产受控联调域名</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
@@ -1276,12 +1347,12 @@
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">例如 staging.example.com；需公网 HTTPS。</t>
+          <t xml:space="preserve">例如 ivybm.com；一期没有常驻 staging，真实 Webhook 仅在获批的 production 受控窗口联调。</t>
         </is>
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H13" s="11" t="inlineStr">
@@ -1323,7 +1394,7 @@
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
@@ -1365,7 +1436,7 @@
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H15" s="11" t="inlineStr">
@@ -1407,7 +1478,7 @@
       </c>
       <c r="G16" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1453,7 +1524,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">可由技术团队代办。请填写资产归属与负责人；没有账号时填“需新建”。</t>
+          <t xml:space="preserve">平台合约区分 facebook-page 与 instagram-professional。状态列只填枚举；App Secret / Verify Token / OAuth Token 真值不写入本表。</t>
         </is>
       </c>
     </row>
@@ -1532,7 +1603,7 @@
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H5" s="11" t="inlineStr">
@@ -1574,7 +1645,7 @@
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
@@ -1591,12 +1662,12 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Facebook Page</t>
+          <t xml:space="preserve">facebook-page</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page 是否已有 / 希望创建的名称</t>
+          <t xml:space="preserve">Facebook Page 是否已有 / 希望创建名称</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
@@ -1611,12 +1682,12 @@
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">现有 Page 请提供 URL；新建请给英文名称。</t>
+          <t xml:space="preserve">账号类型 = facebook-page；现有 Page 填 URL；新建给英文名称。</t>
         </is>
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H7" s="11" t="inlineStr">
@@ -1633,12 +1704,12 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Facebook Page</t>
+          <t xml:space="preserve">facebook-page</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Page 类别、公开电话、地址、简介</t>
+          <t xml:space="preserve">facebook-page 外部 Page ID</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
@@ -1653,12 +1724,12 @@
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">用于创建或补全企业主页。</t>
+          <t xml:space="preserve">创建后补填；只填公开资产 ID，将进入服务器 allowlist。</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
@@ -1675,12 +1746,12 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Instagram</t>
+          <t xml:space="preserve">facebook-page</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Instagram 账号是否已有 / 希望使用的用户名</t>
+          <t xml:space="preserve">facebook-page 授权状态</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
@@ -1695,12 +1766,12 @@
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">一期需转为商业账号并绑定 Facebook Page。</t>
+          <t xml:space="preserve">从枚举中选：未开始,待处理,已连接,已过期,被阻塞,已停用。</t>
         </is>
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H9" s="11" t="inlineStr">
@@ -1717,12 +1788,12 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Instagram</t>
+          <t xml:space="preserve">facebook-page</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">确认可转为商业账号并绑定 Page</t>
+          <t xml:space="preserve">Messenger 内容/订阅授权确认</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
@@ -1737,12 +1808,12 @@
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">填写“确认”或说明限制。</t>
+          <t xml:space="preserve">确认 Page 同意接收 Messenger 与 Webhook 订阅。</t>
         </is>
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
@@ -1759,12 +1830,12 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Meta App</t>
+          <t xml:space="preserve">facebook-page</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">开发者应用名称</t>
+          <t xml:space="preserve">facebook-page 消息入站审批状态</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
@@ -1779,12 +1850,12 @@
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">建议：品牌名 + Messaging。</t>
+          <t xml:space="preserve">枚举：未开始,待审核,已通过,被阻塞；等待 App Review 通过才能进入生产。</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H11" s="11" t="inlineStr">
@@ -1801,12 +1872,12 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Meta App</t>
+          <t xml:space="preserve">facebook-page</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">应用最终管理员姓名 / 企业邮箱</t>
+          <t xml:space="preserve">facebook-page 图文发布审批状态</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
@@ -1821,12 +1892,12 @@
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">负责验证码、权限申请和最终接管。</t>
+          <t xml:space="preserve">枚举：未开始,待审核,已通过,被阻塞；当前一期联调以 PublishJobs / PublishLogs / adapter 评审为准。</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
@@ -1843,12 +1914,12 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Webhook</t>
+          <t xml:space="preserve">instagram-professional</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">预生产回调域名确认</t>
+          <t xml:space="preserve">Instagram 账号是否已有 / 希望使用的用户名</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
@@ -1863,12 +1934,12 @@
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">系统回调路径固定为 /api/webhooks/meta。</t>
+          <t xml:space="preserve">账号类型 = instagram-professional；一期需转为商业账号并绑定 Facebook Page。</t>
         </is>
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H13" s="11" t="inlineStr">
@@ -1885,12 +1956,12 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Webhook</t>
+          <t xml:space="preserve">instagram-professional</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Meta Page ID（创建后补填）</t>
+          <t xml:space="preserve">instagram-professional 外部 Account ID</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
@@ -1905,12 +1976,12 @@
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">将进入服务器 allowlist；只填公开资产 ID。</t>
+          <t xml:space="preserve">创建后补填；只填公开资产 ID，将进入服务器 allowlist。</t>
         </is>
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
@@ -1927,12 +1998,12 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Webhook</t>
+          <t xml:space="preserve">instagram-professional</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Instagram Professional Account ID（创建后补填）</t>
+          <t xml:space="preserve">instagram-professional 授权状态</t>
         </is>
       </c>
       <c r="D15" s="10" t="inlineStr">
@@ -1947,12 +2018,12 @@
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">将进入服务器 allowlist；只填公开资产 ID。</t>
+          <t xml:space="preserve">枚举：未开始,待处理,已连接,已过期,被阻塞,已停用。</t>
         </is>
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H15" s="11" t="inlineStr">
@@ -1969,12 +2040,12 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">联调</t>
+          <t xml:space="preserve">instagram-professional</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">测试发送方 Facebook / Instagram 账号负责人</t>
+          <t xml:space="preserve">instagram-professional 消息入站审批状态</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
@@ -1989,12 +2060,12 @@
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">用于 Development Mode 联调。</t>
+          <t xml:space="preserve">枚举：未开始,待审核,已通过,被阻塞；等待 App Review。</t>
         </is>
       </c>
       <c r="G16" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -2011,12 +2082,12 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">审核</t>
+          <t xml:space="preserve">instagram-professional</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">是否同意提交 App Review 和录制演示</t>
+          <t xml:space="preserve">instagram-professional 图文发布审批状态</t>
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr">
@@ -2031,12 +2102,12 @@
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">生产权限通常需要企业验证、说明与录屏。</t>
+          <t xml:space="preserve">枚举：未开始,待审核,已通过,被阻塞；以 PublishJobs / PublishLogs / adapter 评审为准。</t>
         </is>
       </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H17" s="11" t="inlineStr">
@@ -2053,48 +2124,384 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
+          <t xml:space="preserve">Meta App</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">开发者应用名称</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">必填</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">建议：品牌名 + Messaging。</t>
+        </is>
+      </c>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H18" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未开始</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M-15</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Meta App</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">应用最终管理员姓名 / 企业邮箱</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">必填</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">负责验证码、权限申请和最终接管。</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H19" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未开始</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M-16</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Webhook</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">production 受控回调域名确认</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">必填</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">系统回调路径固定为 /api/webhooks/meta；一期没有常驻 staging。</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未开始</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M-17</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Webhook</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">META_WEBHOOK_ALLOWED_ACCOUNT_IDS allowlist 部署确认</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">必填</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">枚举：待确认,已确认部署,无需部署,被阻塞；只填状态，不填真实 ID 列表。</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H21" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未开始</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M-18</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Webhook</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">META_WEBHOOK_APP_SECRET 部署确认</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">必填</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">枚举：待确认,已确认部署,无需部署,被阻塞；确认 App Secret 已写入服务器受控 storage，绝不写本表。</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H22" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未开始</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M-19</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Webhook</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">META_WEBHOOK_VERIFY_TOKEN 部署确认</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">必填</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">枚举：待确认,已确认部署,无需部署,被阻塞；确认 Verify Token 已写入服务器受控 storage，绝不写本表。</t>
+        </is>
+      </c>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H23" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未开始</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M-20</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">联调</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">测试发送方 Facebook / Instagram 账号负责人</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">必填</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">用于 Development Mode 联调。</t>
+        </is>
+      </c>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H24" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未开始</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M-21</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">审核</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是否同意提交 App Review 和录制演示</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">必填</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">生产权限通常需要企业验证、说明与录屏。</t>
+        </is>
+      </c>
+      <c r="G25" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H25" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未开始</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M-22</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
           <t xml:space="preserve">发布</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="C26" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Facebook / Instagram 图文发布是否纳入一期</t>
         </is>
       </c>
-      <c r="D18" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E18" s="7" t="inlineStr">
+      <c r="D26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">建议</t>
         </is>
       </c>
-      <c r="F18" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">自动发布仍等待内容发布任务结构合并。</t>
-        </is>
-      </c>
-      <c r="G18" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
-        </is>
-      </c>
-      <c r="H18" s="11" t="inlineStr">
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">发布仍以 PublishJobs / PublishLogs / adapter 评审为前置条件；未评审通过不承诺自动联调。</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H26" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">未开始</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H18"/>
+  <autoFilter ref="A4:H26"/>
   <mergeCells count="2">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H5:H18">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H5:H26">
       <formula1>"未开始,已提供,待补充,不适用"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2124,7 +2531,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">个人身份账号必须由真实员工 / 负责人持有；不要创建或转交虚假个人 LinkedIn 账号。</t>
+          <t xml:space="preserve">个人身份账号必须由真实员工 / 负责人持有；区分 linkedin-member 与 linkedin-organization，LinkedIn 私信不在一期范围。</t>
         </is>
       </c>
     </row>
@@ -2178,12 +2585,12 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">个人管理员</t>
+          <t xml:space="preserve">linkedin-member</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">指定 LinkedIn 真实个人管理员姓名 / 企业邮箱</t>
+          <t xml:space="preserve">真实个人管理员姓名 / 企业邮箱</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
@@ -2198,12 +2605,12 @@
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">后续应成为企业主页 Super Admin。</t>
+          <t xml:space="preserve">账号类型 = linkedin-member；必须由真实员工或负责人本人持有。</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H5" s="11" t="inlineStr">
@@ -2220,12 +2627,12 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">个人管理员</t>
+          <t xml:space="preserve">linkedin-member</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">管理员现有 LinkedIn Profile URL 或“需由本人新建”</t>
+          <t xml:space="preserve">linkedin-member Profile URL 与外部 Member ID</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
@@ -2240,12 +2647,12 @@
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">本人需完成 LinkedIn 验证及二次验证。</t>
+          <t xml:space="preserve">现有账号填写 URL / ID；无账号填写“需由本人新建”，不要创建或转交虚假个人账号。</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
@@ -2262,12 +2669,12 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">企业主页</t>
+          <t xml:space="preserve">linkedin-member</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">LinkedIn Company Page URL 或希望创建的英文名</t>
+          <t xml:space="preserve">linkedin-member 授权状态</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
@@ -2282,12 +2689,12 @@
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">新建 Page 需品牌、官网、Logo、简介。</t>
+          <t xml:space="preserve">枚举：未开始,待处理,已连接,已过期,被阻塞,已停用；只填状态，不填 OAuth Token。</t>
         </is>
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H7" s="11" t="inlineStr">
@@ -2304,12 +2711,12 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">企业主页</t>
+          <t xml:space="preserve">linkedin-organization</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">企业主页最终 Super Admin</t>
+          <t xml:space="preserve">企业主页 URL 或希望创建的英文名</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
@@ -2324,12 +2731,12 @@
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">由客户侧负责人保留最高权限。</t>
+          <t xml:space="preserve">账号类型 = linkedin-organization；新建 Page 需品牌、官网、Logo、简介。</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
@@ -2346,12 +2753,12 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Developer App</t>
+          <t xml:space="preserve">linkedin-organization</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">开发者应用名称</t>
+          <t xml:space="preserve">linkedin-organization 外部 Organization ID</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
@@ -2366,12 +2773,12 @@
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">技术团队可代建，资产归客户公司。</t>
+          <t xml:space="preserve">创建后补填；只填公开组织 ID。</t>
         </is>
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H9" s="11" t="inlineStr">
@@ -2388,12 +2795,12 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">OAuth</t>
+          <t xml:space="preserve">linkedin-organization</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">允许使用的 HTTPS 回调域名</t>
+          <t xml:space="preserve">linkedin-organization 授权状态</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
@@ -2408,12 +2815,12 @@
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">用于 LinkedIn OAuth redirect URL。</t>
+          <t xml:space="preserve">枚举：未开始,待处理,已连接,已过期,被阻塞,已停用；只填状态，不填 OAuth Token。</t>
         </is>
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
@@ -2430,12 +2837,12 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">发布范围</t>
+          <t xml:space="preserve">企业主页</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">需要个人发帖、企业主页发帖，或两者</t>
+          <t xml:space="preserve">客户侧最终 Super Admin</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
@@ -2450,12 +2857,12 @@
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">两类权限与审核要求不同。</t>
+          <t xml:space="preserve">由客户侧负责人保留最高权限，技术团队只保留获授权的有限角色。</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H11" s="11" t="inlineStr">
@@ -2472,12 +2879,12 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">审核</t>
+          <t xml:space="preserve">Developer App</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">是否同意申请 Marketing / Community Management 权限</t>
+          <t xml:space="preserve">开发者应用名称与最终管理员</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
@@ -2485,19 +2892,19 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">建议</t>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">必填</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">企业主页自动发帖通常需要额外权限。</t>
+          <t xml:space="preserve">技术团队可协助创建，资产和最终控制权归客户公司。</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
@@ -2514,48 +2921,174 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
+          <t xml:space="preserve">OAuth</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">生产 HTTPS 回调域名</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">必填</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">用于 LinkedIn OAuth redirect URL；一期没有常驻 staging。</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H13" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未开始</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L-10</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">发布权限</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">个人 / 企业主页发布 API 审批状态</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">必填</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">枚举：未开始,待审核,已通过,被阻塞；LinkedIn API 未获批时使用审核、素材清单和复制文案的辅助导出。</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H14" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未开始</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L-11</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">发布范围</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">需要个人发帖、企业主页发帖，或两者</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">必填</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">两类权限与审核要求不同。</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H15" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未开始</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L-12</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
           <t xml:space="preserve">联调</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">可用于测试发布的企业主页 / 审核人</t>
         </is>
       </c>
-      <c r="D13" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">建议</t>
         </is>
       </c>
-      <c r="F13" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">测试内容发布前需客户确认。</t>
-        </is>
-      </c>
-      <c r="G13" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
-        </is>
-      </c>
-      <c r="H13" s="11" t="inlineStr">
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">测试内容发布前需客户确认；未获权限不承诺自动发布。</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H16" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">未开始</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H13"/>
+  <autoFilter ref="A4:H16"/>
   <mergeCells count="2">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H5:H13">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H5:H16">
       <formula1>"未开始,已提供,待补充,不适用"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2585,7 +3118,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TikTok 私信 API 受目标地区、商业账号资格和官方审核影响；本表用于资格确认，不承诺自动接入一定可用。</t>
+          <t xml:space="preserve">TikTok 私信 API 受目标地区、商业账号资格、官方 schema 与审核影响；当前仅记录阻塞与申请状态，不承诺自动接入。</t>
         </is>
       </c>
     </row>
@@ -2639,7 +3172,7 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">商业账号</t>
+          <t xml:space="preserve">tiktok-business</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -2659,12 +3192,12 @@
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">提供链接 / ID 或填写“需新建”。</t>
+          <t xml:space="preserve">账号类型 = tiktok-business；提供链接或填写“需新建”。</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H5" s="11" t="inlineStr">
@@ -2681,12 +3214,12 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">商业账号</t>
+          <t xml:space="preserve">tiktok-business</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Business Account 最终 Owner 姓名 / 企业邮箱</t>
+          <t xml:space="preserve">tiktok-business 外部 Account ID</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
@@ -2701,12 +3234,12 @@
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">客户保留最高管理员。</t>
+          <t xml:space="preserve">创建后补填；只填公开账号 ID。</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
@@ -2723,12 +3256,12 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">地区</t>
+          <t xml:space="preserve">tiktok-business</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">目标运营国家 / 地区</t>
+          <t xml:space="preserve">tiktok-business 授权状态</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
@@ -2743,12 +3276,12 @@
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">决定 Business Messaging API 的可用性。</t>
+          <t xml:space="preserve">枚举：未开始,待处理,已连接,已过期,被阻塞,已停用；只填状态，不填 access token。</t>
         </is>
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H7" s="11" t="inlineStr">
@@ -2765,12 +3298,12 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">主体</t>
+          <t xml:space="preserve">商业账号</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">是否可提供企业认证资料</t>
+          <t xml:space="preserve">Business Account 最终 Owner 姓名 / 企业邮箱</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
@@ -2785,12 +3318,12 @@
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通常需营业执照、主体名称、地址等。</t>
+          <t xml:space="preserve">客户保留最高管理员和恢复方式。</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
@@ -2807,12 +3340,12 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">开发者</t>
+          <t xml:space="preserve">地区</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">TikTok for Developers 账号是否已有 / 需新建</t>
+          <t xml:space="preserve">目标运营国家 / 地区</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
@@ -2827,12 +3360,12 @@
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">技术团队可代建。</t>
+          <t xml:space="preserve">决定官方能力是否可能开放。</t>
         </is>
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H9" s="11" t="inlineStr">
@@ -2849,12 +3382,12 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">资格</t>
+          <t xml:space="preserve">主体</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">是否已有 TikTok 客户经理 / 支持工单</t>
+          <t xml:space="preserve">是否可提供企业认证资料</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
@@ -2862,19 +3395,19 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">建议</t>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">必填</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">请提供联系人或工单号，不要提供密码。</t>
+          <t xml:space="preserve">通常需营业执照、主体名称、地址等；证件通过受控方式提供。</t>
         </is>
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
@@ -2891,12 +3424,12 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">资格</t>
+          <t xml:space="preserve">开发者</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">官方是否确认该地区可用商业私信入站 API</t>
+          <t xml:space="preserve">TikTok for Developers 账号是否已有 / 需新建</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
@@ -2911,12 +3444,12 @@
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">未确认则保持 blocked，不创建猜测接口。</t>
+          <t xml:space="preserve">技术团队可协助，客户保留最终管理员。</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H11" s="11" t="inlineStr">
@@ -2933,48 +3466,174 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
+          <t xml:space="preserve">资格</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TikTok 客户经理 / 官方支持工单</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">建议</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">提供联系人或工单号，不要提供密码。</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H12" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未开始</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T-09</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">官方 schema</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">私信入站 event schema 官方证据状态</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">必填</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当前口径：待官方确认,被阻塞,暂不可用；填写官方文档链接、工单号或“待官方确认”，未确认时保持 blocked。</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H13" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未开始</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T-10</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API 资格</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">目标地区与商业账号私信 API eligibility 状态</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">必填</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">当前口径：待官方确认,被阻塞,暂不可用；未通过不得要求实现猜测 payload 或自动接入。</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H14" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未开始</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T-11</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
           <t xml:space="preserve">联调</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">测试 TikTok 商业账号与测试人员</t>
         </is>
       </c>
-      <c r="D12" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">建议</t>
         </is>
       </c>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">资格确认后再安排。</t>
-        </is>
-      </c>
-      <c r="G12" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
-        </is>
-      </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">仅在官方 schema 与资格均确认后安排受控联调。</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H15" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">未开始</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H12"/>
+  <autoFilter ref="A4:H15"/>
   <mergeCells count="2">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H5:H12">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H5:H15">
       <formula1>"未开始,已提供,待补充,不适用"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3004,7 +3663,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">本页用于安排域名、受控 secret 注入、审核材料和资产交接；不要填写任何真实 secret。</t>
+          <t xml:space="preserve">本页用于安排 production 受控联调、受控 secret 注入、审核材料和资产交接；一期没有常驻 staging，不要填写任何真实 secret。</t>
         </is>
       </c>
     </row>
@@ -3063,7 +3722,7 @@
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">预生产环境负责人 / 联系方式</t>
+          <t xml:space="preserve">production 受控联调负责人 / 联系方式</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
@@ -3078,12 +3737,12 @@
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">用于公开 HTTPS 回调联调。</t>
+          <t xml:space="preserve">真实 Webhook 与平台操作只在获批的 production 窗口执行。</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H5" s="11" t="inlineStr">
@@ -3120,12 +3779,12 @@
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">生产发布与 secret 注入需授权。</t>
+          <t xml:space="preserve">生产发布、secret 注入与账号授权需由其确认。</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
@@ -3162,12 +3821,12 @@
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">用于 staging / production 域名和 HTTPS。</t>
+          <t xml:space="preserve">用于 production 域名、HTTPS 与平台回调校验；一期没有常驻 staging。</t>
         </is>
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H7" s="11" t="inlineStr">
@@ -3189,7 +3848,7 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">确认 Meta App Secret 与 verify token 只写入服务器</t>
+          <t xml:space="preserve">Meta allowlist / App Secret / Verify Token 服务器部署确认</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
@@ -3204,12 +3863,12 @@
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">填写“确认”；不要在 Excel 填实际值。</t>
+          <t xml:space="preserve">枚举：待确认,已确认部署,无需部署,被阻塞；只填状态，绝不填真实值。</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
@@ -3226,12 +3885,12 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">审核</t>
+          <t xml:space="preserve">Secret</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">App Review 业务用途说明负责人</t>
+          <t xml:space="preserve">平台 OAuth / access token 受控注入确认</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
@@ -3246,12 +3905,12 @@
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">需说明客户如何使用消息和发布能力。</t>
+          <t xml:space="preserve">枚举：待确认,已确认部署,无需部署,被阻塞；token 只进入服务器受控 storage，不经 Excel、聊天或 PR 传递。</t>
         </is>
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H9" s="11" t="inlineStr">
@@ -3273,7 +3932,7 @@
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">可提供审核录屏 / 截图的联系人</t>
+          <t xml:space="preserve">App Review 业务用途说明负责人</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
@@ -3288,12 +3947,12 @@
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Meta / LinkedIn 可能要求。</t>
+          <t xml:space="preserve">需说明客户如何使用消息和发布能力。</t>
         </is>
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
@@ -3310,12 +3969,12 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">内容</t>
+          <t xml:space="preserve">审核</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">测试消息与测试发布内容确认人</t>
+          <t xml:space="preserve">可提供审核录屏 / 截图的联系人</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
@@ -3330,12 +3989,12 @@
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">避免未经确认的公开发布。</t>
+          <t xml:space="preserve">Meta / LinkedIn 可能要求。</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H11" s="11" t="inlineStr">
@@ -3352,12 +4011,12 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">交接</t>
+          <t xml:space="preserve">内容</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">客户最终接收企业邮箱、2FA、管理员权限的人</t>
+          <t xml:space="preserve">测试消息与测试发布内容确认人</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
@@ -3372,12 +4031,12 @@
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">账号开通后由其改密并保留恢复方式。</t>
+          <t xml:space="preserve">避免未经确认的公开发布。</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
@@ -3399,7 +4058,7 @@
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">技术团队保留的角色与有效期</t>
+          <t xml:space="preserve">客户最终接收企业邮箱、2FA、管理员权限的人</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
@@ -3407,19 +4066,19 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">建议</t>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">必填</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">例如 Developer / Technical admin，便于后续维护。</t>
+          <t xml:space="preserve">账号开通后由其改密并保留恢复方式。</t>
         </is>
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
         </is>
       </c>
       <c r="H13" s="11" t="inlineStr">
@@ -3436,48 +4095,90 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
+          <t xml:space="preserve">交接</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">技术团队保留的角色与有效期</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">建议</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">例如 Developer / Technical admin，便于后续维护。</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H14" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未开始</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H-11</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
           <t xml:space="preserve">确认</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">客户确认不向技术团队索要 / 提供密码、token、银行卡</t>
         </is>
       </c>
-      <c r="D14" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">必填</t>
-        </is>
-      </c>
-      <c r="F14" s="9" t="inlineStr">
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">必填</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">填写“确认”。</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、App Secret、OAuth Token 或银行卡信息。</t>
-        </is>
-      </c>
-      <c r="H14" s="11" t="inlineStr">
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H15" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">未开始</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H14"/>
+  <autoFilter ref="A4:H15"/>
   <mergeCells count="2">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H5:H14">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H5:H15">
       <formula1>"未开始,已提供,待补充,不适用"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
docs(task-13): harden accountless onboarding pack
</commit_message>
<xml_diff>
--- a/docs/client-materials/IVYBM_海外平台账号申请资料收集表.xlsx
+++ b/docs/client-materials/IVYBM_海外平台账号申请资料收集表.xlsx
@@ -167,7 +167,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">文档版本：2026-07-25    最后更新：2026-07-25    适用范围：海外平台账号申请资料收集（客户侧、非密）</t>
+          <t xml:space="preserve">文档版本：2026-07-26    最后更新：2026-07-26    适用范围：海外平台账号申请资料收集（客户侧、非密）</t>
         </is>
       </c>
     </row>
@@ -188,7 +188,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">2. 企业主体、品牌、页面和开发者应用最终归客户公司所有；请指定可接收验证码并完成最终接管的负责人。</t>
+          <t xml:space="preserve">2. 企业主体、品牌、业务账号和主页最终归客户公司所有；开发者 App 的归属按平台与书面授权确认：默认 Meta 使用 IVYBM 受控 App，TikTok / LinkedIn 仅在对应路径确认后由客户自持。</t>
         </is>
       </c>
     </row>
@@ -237,7 +237,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">排除：WhatsApp 不进入一期系统接入；LinkedIn 私信不属于一期自动接入范围。</t>
+          <t xml:space="preserve">排除：WhatsApp 不进入一期系统接入；LinkedIn 私信不属于一期自动接入范围；TikTok 图文发布不在一期范围。</t>
         </is>
       </c>
     </row>
@@ -265,7 +265,7 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TikTok：tiktok-business 填写外部账号 ID、授权状态；私信 schema 与 API 资格当前统一标记为“被阻塞 / 待官方确认”，订单前再次确认，不承诺自动接入。</t>
+          <t xml:space="preserve">TikTok：tiktok-business 填写外部账号 ID、授权状态；私信 schema 与 API 资格当前统一标记为“待官方确认（conditional）/ 被阻塞（blocked）”，不承诺自动接入。</t>
         </is>
       </c>
     </row>
@@ -300,7 +300,7 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">审批状态枚举：未开始、待审核、已通过、被阻塞。</t>
+          <t xml:space="preserve">审批状态枚举：未开始、待审核、已通过、被阻塞。注意：审批“已通过”仅表示平台审核状态，不等于已在真实受控环境验证为 available。</t>
         </is>
       </c>
     </row>
@@ -314,7 +314,7 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">TikTok 私信当前口径枚举：待官方确认、被阻塞、暂不可用。</t>
+          <t xml:space="preserve">TikTok 私信当前口径枚举：待官方确认（conditional）、被阻塞（blocked）。</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">用于验证码 / 二次验证；不要写密码。</t>
+          <t xml:space="preserve">用于验证码 / 二次验证；仅通过受控文件夹或指定企业账号单聊提供，不要写密码。</t>
         </is>
       </c>
       <c r="G14" s="9" t="inlineStr">
@@ -907,7 +907,7 @@
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H5:H16">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16">
       <formula1>"未开始,已提供,待补充,不适用"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1347,7 +1347,7 @@
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">例如 ivybm.com；一期没有常驻 staging，真实 Webhook 仅在获批的 production 受控窗口联调。</t>
+          <t xml:space="preserve">例如 client-domain.com；通常为客户官网同域。一期没有常驻 staging，真实 Webhook 仅在获批的 production 受控窗口联调。</t>
         </is>
       </c>
       <c r="G13" s="9" t="inlineStr">
@@ -1494,7 +1494,7 @@
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H5:H16">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16">
       <formula1>"未开始,已提供,待补充,不适用"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">开发者应用名称</t>
+          <t xml:space="preserve">Meta App 归属路径</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
@@ -2144,7 +2144,7 @@
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">建议：品牌名 + Messaging。</t>
+          <t xml:space="preserve">默认填写“IVYBM 受控 App”；只有合同或 IVYBM 书面操作单明确要求时才填写“客户自持 App”。</t>
         </is>
       </c>
       <c r="G18" s="9" t="inlineStr">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">应用最终管理员姓名 / 企业邮箱</t>
+          <t xml:space="preserve">客户自持 Meta App 名称</t>
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr">
@@ -2181,12 +2181,12 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">必填</t>
+          <t xml:space="preserve">条件必填</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">负责验证码、权限申请和最终接管。</t>
+          <t xml:space="preserve">仅在 M-14 选择“客户自持 App”时填写；默认 IVYBM 受控 App 路径填“不适用”。</t>
         </is>
       </c>
       <c r="G19" s="9" t="inlineStr">
@@ -2208,12 +2208,12 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Webhook</t>
+          <t xml:space="preserve">Meta App</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">production 受控回调域名确认</t>
+          <t xml:space="preserve">客户自持 Meta App 最终管理员姓名 / 企业邮箱</t>
         </is>
       </c>
       <c r="D20" s="10" t="inlineStr">
@@ -2223,12 +2223,12 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">必填</t>
+          <t xml:space="preserve">条件必填</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">系统回调路径固定为 /api/webhooks/meta；一期没有常驻 staging。</t>
+          <t xml:space="preserve">仅客户自持 App 时填写；不得要求客户登录或接管 IVYBM 受控 App。</t>
         </is>
       </c>
       <c r="G20" s="9" t="inlineStr">
@@ -2255,7 +2255,7 @@
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">META_WEBHOOK_ALLOWED_ACCOUNT_IDS allowlist 部署确认</t>
+          <t xml:space="preserve">production 受控回调域名确认</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
@@ -2270,7 +2270,7 @@
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">枚举：待确认,已确认部署,无需部署,被阻塞；只填状态，不填真实 ID 列表。</t>
+          <t xml:space="preserve">系统回调路径固定为 /api/webhooks/meta；一期没有常驻 staging。</t>
         </is>
       </c>
       <c r="G21" s="9" t="inlineStr">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">META_WEBHOOK_APP_SECRET 部署确认</t>
+          <t xml:space="preserve">META_WEBHOOK_ALLOWED_ACCOUNT_IDS allowlist 部署确认</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
@@ -2312,7 +2312,7 @@
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">枚举：待确认,已确认部署,无需部署,被阻塞；确认 App Secret 已写入服务器受控 storage，绝不写本表。</t>
+          <t xml:space="preserve">枚举：待确认,已确认部署,无需部署,被阻塞；只填状态，不填真实 ID 列表。</t>
         </is>
       </c>
       <c r="G22" s="9" t="inlineStr">
@@ -2322,7 +2322,7 @@
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">未开始</t>
+          <t xml:space="preserve">待确认</t>
         </is>
       </c>
     </row>
@@ -2339,7 +2339,7 @@
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">META_WEBHOOK_VERIFY_TOKEN 部署确认</t>
+          <t xml:space="preserve">META_WEBHOOK_APP_SECRET 部署确认</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
@@ -2354,7 +2354,7 @@
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">枚举：待确认,已确认部署,无需部署,被阻塞；确认 Verify Token 已写入服务器受控 storage，绝不写本表。</t>
+          <t xml:space="preserve">枚举：待确认,已确认部署,无需部署,被阻塞；确认 App Secret 已写入服务器受控 storage，绝不写本表。</t>
         </is>
       </c>
       <c r="G23" s="9" t="inlineStr">
@@ -2364,7 +2364,7 @@
       </c>
       <c r="H23" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">未开始</t>
+          <t xml:space="preserve">待确认</t>
         </is>
       </c>
     </row>
@@ -2376,12 +2376,12 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">联调</t>
+          <t xml:space="preserve">Webhook</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">测试发送方 Facebook / Instagram 账号负责人</t>
+          <t xml:space="preserve">META_WEBHOOK_VERIFY_TOKEN 部署确认</t>
         </is>
       </c>
       <c r="D24" s="10" t="inlineStr">
@@ -2396,7 +2396,7 @@
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">用于 Development Mode 联调。</t>
+          <t xml:space="preserve">枚举：待确认,已确认部署,无需部署,被阻塞；确认 Verify Token 已写入服务器受控 storage，绝不写本表。</t>
         </is>
       </c>
       <c r="G24" s="9" t="inlineStr">
@@ -2406,7 +2406,7 @@
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">未开始</t>
+          <t xml:space="preserve">待确认</t>
         </is>
       </c>
     </row>
@@ -2418,12 +2418,12 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">审核</t>
+          <t xml:space="preserve">联调</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">是否同意提交 App Review 和录制演示</t>
+          <t xml:space="preserve">测试发送方 Facebook / Instagram 账号负责人</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">生产权限通常需要企业验证、说明与录屏。</t>
+          <t xml:space="preserve">用于 Development Mode 联调。</t>
         </is>
       </c>
       <c r="G25" s="9" t="inlineStr">
@@ -2460,49 +2460,100 @@
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
+          <t xml:space="preserve">审核</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是否同意提交 App Review 和录制演示</t>
+        </is>
+      </c>
+      <c r="D26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">必填</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">生产权限通常需要企业验证、说明与录屏。</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H26" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未开始</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M-23</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
           <t xml:space="preserve">发布</t>
         </is>
       </c>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Facebook / Instagram 图文发布是否纳入一期</t>
-        </is>
-      </c>
-      <c r="D26" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E26" s="7" t="inlineStr">
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Facebook / Instagram 图文发布受控测试意向</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">建议</t>
         </is>
       </c>
-      <c r="F26" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">发布仍以 PublishJobs / PublishLogs / adapter 评审为前置条件；未评审通过不承诺自动联调。</t>
-        </is>
-      </c>
-      <c r="G26" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
-        </is>
-      </c>
-      <c r="H26" s="11" t="inlineStr">
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">不改变一期冻结范围；发布仍以 PublishJobs / PublishLogs / adapter 评审为前置条件，未评审通过不承诺自动联调。</t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H27" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">未开始</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H26"/>
+  <autoFilter ref="A4:H27"/>
   <mergeCells count="2">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H5:H26">
+  <dataValidations count="4">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H10 H13 H14 H18 H19 H20 H21 H25 H26 H27">
       <formula1>"未开始,已提供,待补充,不适用"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H9 H15">
+      <formula1>"未开始,待处理,已连接,已过期,被阻塞,已停用"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H11 H12 H16 H17">
+      <formula1>"未开始,待审核,已通过,被阻塞"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H22 H23 H24">
+      <formula1>"待确认,已确认部署,无需部署,被阻塞"</formula1>
     </dataValidation>
   </dataValidations>
 </worksheet>
@@ -2884,7 +2935,7 @@
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">开发者应用名称与最终管理员</t>
+          <t xml:space="preserve">客户自持 Developer App 名称与最终管理员</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
@@ -2894,12 +2945,12 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">必填</t>
+          <t xml:space="preserve">条件必填</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">技术团队可协助创建，资产和最终控制权归客户公司。</t>
+          <t xml:space="preserve">仅在 IVYBM 书面确认采用客户自持 App 或企业主页自动发布路径时填写；个人账号受控 App 路径填“不适用”。</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
@@ -2926,7 +2977,7 @@
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">生产 HTTPS 回调域名</t>
+          <t xml:space="preserve">客户自持 App 的生产 HTTPS 回调域名</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
@@ -2936,12 +2987,12 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">必填</t>
+          <t xml:space="preserve">条件必填</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">用于 LinkedIn OAuth redirect URL；一期没有常驻 staging。</t>
+          <t xml:space="preserve">仅客户自持 App 时填写，用于 LinkedIn OAuth redirect URL；一期没有常驻 staging。</t>
         </is>
       </c>
       <c r="G13" s="9" t="inlineStr">
@@ -3087,9 +3138,15 @@
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H5:H16">
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H5 H6 H8 H9 H11 H12 H13 H15 H16">
       <formula1>"未开始,已提供,待补充,不适用"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H7 H10">
+      <formula1>"未开始,待处理,已连接,已过期,被阻塞,已停用"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H14">
+      <formula1>"未开始,待审核,已通过,被阻塞"</formula1>
     </dataValidation>
   </dataValidations>
 </worksheet>
@@ -3439,12 +3496,12 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">必填</t>
+          <t xml:space="preserve">条件必填</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">技术团队可协助，客户保留最终管理员。</t>
+          <t xml:space="preserve">仅在 TikTok-3 私信资格决策门已有“可申请”或“已批准”证据后填写；技术团队可协助，客户保留最终管理员。</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
@@ -3528,7 +3585,7 @@
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">当前口径：待官方确认,被阻塞,暂不可用；填写官方文档链接、工单号或“待官方确认”，未确认时保持 blocked。</t>
+          <t xml:space="preserve">当前口径：待官方确认（conditional）,被阻塞（blocked）；填写官方文档链接、工单号或“待官方确认”，未确认时保持 blocked。</t>
         </is>
       </c>
       <c r="G13" s="9" t="inlineStr">
@@ -3538,7 +3595,7 @@
       </c>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">未开始</t>
+          <t xml:space="preserve">被阻塞（blocked）</t>
         </is>
       </c>
     </row>
@@ -3570,7 +3627,7 @@
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">当前口径：待官方确认,被阻塞,暂不可用；未通过不得要求实现猜测 payload 或自动接入。</t>
+          <t xml:space="preserve">当前口径：待官方确认（conditional）,被阻塞（blocked）；未通过不得要求实现猜测 payload 或自动接入。</t>
         </is>
       </c>
       <c r="G14" s="9" t="inlineStr">
@@ -3580,7 +3637,7 @@
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">未开始</t>
+          <t xml:space="preserve">被阻塞（blocked）</t>
         </is>
       </c>
     </row>
@@ -3632,9 +3689,15 @@
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H5:H15">
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H5 H6 H8 H9 H10 H11 H12 H15">
       <formula1>"未开始,已提供,待补充,不适用"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H7">
+      <formula1>"未开始,待处理,已连接,已过期,被阻塞,已停用"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H13 H14">
+      <formula1>"待官方确认（conditional）,被阻塞（blocked）"</formula1>
     </dataValidation>
   </dataValidations>
 </worksheet>
@@ -3873,7 +3936,7 @@
       </c>
       <c r="H8" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">未开始</t>
+          <t xml:space="preserve">待确认</t>
         </is>
       </c>
     </row>
@@ -3915,7 +3978,7 @@
       </c>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">未开始</t>
+          <t xml:space="preserve">待确认</t>
         </is>
       </c>
     </row>
@@ -4171,15 +4234,228 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H-12</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">授权记录</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">授权申请 / 变更记录编号</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">建议</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">仅填工单、邮件或审批记录编号，不填授权码、密码或 token。</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H16" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未开始</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H-13</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">授权记录</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">授权生效日、到期日或下次复核日</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">建议</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">记录可撤销授权的有效期；日期可后补。</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H17" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未开始</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H-14</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">撤销</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">撤销入口与回收负责人</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">建议</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">例如对应平台的人员/合作伙伴/开发者权限入口及客户侧回收负责人。</t>
+        </is>
+      </c>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H18" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未开始</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H-15</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Secret 记录</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">secret 部署 / 轮换记录编号、执行人、复核人</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">建议</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">仅填受控部署记录编号和角色，不填任何 secret 或 token 真值。</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H19" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未开始</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H-16</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">受控交付</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">双方确认的交付渠道、访问范围、保留 / 清理负责人</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">建议</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">例如受控文件夹路径类别、成员范围、到期清理负责人；不填公开链接或敏感内容。</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未开始</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:H15"/>
+  <autoFilter ref="A4:H20"/>
   <mergeCells count="2">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H5:H15">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H5 H6 H7 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20">
       <formula1>"未开始,已提供,待补充,不适用"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H8 H9">
+      <formula1>"待确认,已确认部署,无需部署,被阻塞"</formula1>
     </dataValidation>
   </dataValidations>
 </worksheet>

</xml_diff>

<commit_message>
docs(task-13): harden client account onboarding pack
</commit_message>
<xml_diff>
--- a/docs/client-materials/IVYBM_海外平台账号申请资料收集表.xlsx
+++ b/docs/client-materials/IVYBM_海外平台账号申请资料收集表.xlsx
@@ -181,7 +181,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. 没有现成账号时，请在对应工作表填写“需新建”及希望使用的账号名；技术团队代为开设与配置。</t>
+          <t xml:space="preserve">1. 没有现成账号时，由客户自行注册/创建并保留最终管理员；在对应工作表填写“需新建”及拟用账号名。IVYBM 仅在收到书面授权和前置条件满足后，协助 API/Webhook/App 配置、审核材料与受控联调，不代注册、养号或恢复账号。</t>
         </is>
       </c>
     </row>
@@ -202,7 +202,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">4. 所有“必填”项会影响账号创建、App Review 或真实联调；“建议”项可后补，但会延长审核时间。</t>
+          <t xml:space="preserve">4. 所有“必填”项会影响客户资产准备、App Review 或真实联调；“建议”项可后补，但会延长审核时间。</t>
         </is>
       </c>
     </row>
@@ -871,7 +871,7 @@
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">书面授权确认人及日期</t>
+          <t xml:space="preserve">书面授权确认人、日期与范围</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
@@ -886,7 +886,7 @@
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">确认可代办平台账号、开发者应用和审核。</t>
+          <t xml:space="preserve">确认客户已创建/将自行创建账号与资产；前置条件满足后，是否书面授权 IVYBM 仅协助 API/Webhook/App 配置及 App Review 技术材料/提交（不含账号注册、养号或恢复）。</t>
         </is>
       </c>
       <c r="G16" s="9" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Meta Business 是否已有 / 需新建</t>
+          <t xml:space="preserve">Meta Business 是否已有 / 需由客户新建</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
@@ -1598,7 +1598,7 @@
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">填写链接或“需新建”。</t>
+          <t xml:space="preserve">填写链接；无账号由客户创建并保留最终 Owner，IVYBM 仅在书面授权后协助集成配置。</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
@@ -1667,7 +1667,7 @@
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Facebook Page 是否已有 / 希望创建名称</t>
+          <t xml:space="preserve">Facebook Page 是否已有 / 客户拟用名称</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">账号类型 = facebook-page；现有 Page 填 URL；新建给英文名称。</t>
+          <t xml:space="preserve">账号类型 = facebook-page；现有 Page 填 URL；无 Page 由客户创建并保留最高管理员。</t>
         </is>
       </c>
       <c r="G7" s="9" t="inlineStr">
@@ -1724,7 +1724,7 @@
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">创建后补填；只填公开资产 ID，将进入服务器 allowlist。</t>
+          <t xml:space="preserve">客户创建/取得后补填；只填公开资产 ID，将进入服务器 allowlist。</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
@@ -1793,7 +1793,7 @@
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Messenger 内容/订阅授权确认</t>
+          <t xml:space="preserve">Facebook Page 消息/内容/管理相关 task 已就绪</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">确认 Page 同意接收 Messenger 与 Webhook 订阅。</t>
+          <t xml:space="preserve">由客户管理员核对用于授权的 Page task；只记录状态与脱敏证据位置，不填 token。</t>
         </is>
       </c>
       <c r="G10" s="9" t="inlineStr">
@@ -1825,7 +1825,7 @@
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">M-07</t>
+          <t xml:space="preserve">M-06A</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">facebook-page 消息入站审批状态</t>
+          <t xml:space="preserve">facebook-page Page task 权限证据（截图/工单编号/受控路径）</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
@@ -1850,7 +1850,7 @@
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">枚举：未开始,待审核,已通过,被阻塞；等待 App Review 通过才能进入生产。</t>
+          <t xml:space="preserve">提供消息、内容、管理/审核 task 的脱敏证据；只填文件名、记录编号或受控路径。</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
@@ -1867,7 +1867,7 @@
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">M-08</t>
+          <t xml:space="preserve">M-07</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
@@ -1877,7 +1877,7 @@
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">facebook-page 图文发布审批状态</t>
+          <t xml:space="preserve">facebook-page 消息入站审批状态</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
@@ -1892,7 +1892,7 @@
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">枚举：未开始,待审核,已通过,被阻塞；当前一期联调以 PublishJobs / PublishLogs / adapter 评审为准。</t>
+          <t xml:space="preserve">枚举：未开始,待审核,已通过,被阻塞；等待 App Review 通过才能进入生产。</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
@@ -1909,17 +1909,17 @@
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">M-09</t>
+          <t xml:space="preserve">M-08</t>
         </is>
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">instagram-professional</t>
+          <t xml:space="preserve">facebook-page</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Instagram 账号是否已有 / 希望使用的用户名</t>
+          <t xml:space="preserve">facebook-page 图文发布审批状态</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
@@ -1934,7 +1934,7 @@
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">账号类型 = instagram-professional；一期需转为商业账号并绑定 Facebook Page。</t>
+          <t xml:space="preserve">枚举：未开始,待审核,已通过,被阻塞；当前一期联调以 PublishJobs / PublishLogs / adapter 评审为准。</t>
         </is>
       </c>
       <c r="G13" s="9" t="inlineStr">
@@ -1951,7 +1951,7 @@
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">M-10</t>
+          <t xml:space="preserve">M-09</t>
         </is>
       </c>
       <c r="B14" s="9" t="inlineStr">
@@ -1961,7 +1961,7 @@
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">instagram-professional 外部 Account ID</t>
+          <t xml:space="preserve">Instagram 账号是否已有 / 客户拟用用户名</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
@@ -1976,7 +1976,7 @@
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">创建后补填；只填公开资产 ID，将进入服务器 allowlist。</t>
+          <t xml:space="preserve">账号类型 = instagram-professional；客户自行创建或转换为商业账号并绑定 Facebook Page。</t>
         </is>
       </c>
       <c r="G14" s="9" t="inlineStr">
@@ -1993,7 +1993,7 @@
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">M-11</t>
+          <t xml:space="preserve">M-10</t>
         </is>
       </c>
       <c r="B15" s="9" t="inlineStr">
@@ -2003,7 +2003,7 @@
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">instagram-professional 授权状态</t>
+          <t xml:space="preserve">instagram-professional 外部 Account ID</t>
         </is>
       </c>
       <c r="D15" s="10" t="inlineStr">
@@ -2018,7 +2018,7 @@
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">枚举：未开始,待处理,已连接,已过期,被阻塞,已停用。</t>
+          <t xml:space="preserve">客户创建/取得后补填；只填公开资产 ID，将进入服务器 allowlist。</t>
         </is>
       </c>
       <c r="G15" s="9" t="inlineStr">
@@ -2035,7 +2035,7 @@
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">M-12</t>
+          <t xml:space="preserve">M-11</t>
         </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
@@ -2045,7 +2045,7 @@
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">instagram-professional 消息入站审批状态</t>
+          <t xml:space="preserve">instagram-professional 授权状态</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
@@ -2060,7 +2060,7 @@
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">枚举：未开始,待审核,已通过,被阻塞；等待 App Review。</t>
+          <t xml:space="preserve">枚举：未开始,待处理,已连接,已过期,被阻塞,已停用。</t>
         </is>
       </c>
       <c r="G16" s="9" t="inlineStr">
@@ -2077,7 +2077,7 @@
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">M-13</t>
+          <t xml:space="preserve">M-12</t>
         </is>
       </c>
       <c r="B17" s="9" t="inlineStr">
@@ -2087,7 +2087,7 @@
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">instagram-professional 图文发布审批状态</t>
+          <t xml:space="preserve">instagram-professional 消息入站审批状态</t>
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">枚举：未开始,待审核,已通过,被阻塞；以 PublishJobs / PublishLogs / adapter 评审为准。</t>
+          <t xml:space="preserve">枚举：未开始,待审核,已通过,被阻塞；等待 App Review。</t>
         </is>
       </c>
       <c r="G17" s="9" t="inlineStr">
@@ -2119,17 +2119,17 @@
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">M-14</t>
+          <t xml:space="preserve">M-12A</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Meta App</t>
+          <t xml:space="preserve">instagram-professional</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Meta App 归属路径</t>
+          <t xml:space="preserve">“允许访问消息 / Allow access to messages”证据（截图/记录编号/日期）</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
@@ -2139,12 +2139,12 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">必填</t>
+          <t xml:space="preserve">条件必填</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">默认填写“IVYBM 受控 App”；只有合同或 IVYBM 书面操作单明确要求时才填写“客户自持 App”。</t>
+          <t xml:space="preserve">当前账号/登录路径显示该开关时，由客户开启并提供脱敏证据；若未显示，提供当前页面截图并标记待官方确认。</t>
         </is>
       </c>
       <c r="G18" s="9" t="inlineStr">
@@ -2161,17 +2161,17 @@
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">M-15</t>
+          <t xml:space="preserve">M-13</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Meta App</t>
+          <t xml:space="preserve">instagram-professional</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">客户自持 Meta App 名称</t>
+          <t xml:space="preserve">instagram-professional 图文发布审批状态</t>
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr">
@@ -2181,12 +2181,12 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">条件必填</t>
+          <t xml:space="preserve">必填</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">仅在 M-14 选择“客户自持 App”时填写；默认 IVYBM 受控 App 路径填“不适用”。</t>
+          <t xml:space="preserve">枚举：未开始,待审核,已通过,被阻塞；以 PublishJobs / PublishLogs / adapter 评审为准。</t>
         </is>
       </c>
       <c r="G19" s="9" t="inlineStr">
@@ -2203,7 +2203,7 @@
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">M-16</t>
+          <t xml:space="preserve">M-14</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
@@ -2213,7 +2213,7 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">客户自持 Meta App 最终管理员姓名 / 企业邮箱</t>
+          <t xml:space="preserve">Meta App 归属路径</t>
         </is>
       </c>
       <c r="D20" s="10" t="inlineStr">
@@ -2223,12 +2223,12 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">条件必填</t>
+          <t xml:space="preserve">必填</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">仅客户自持 App 时填写；不得要求客户登录或接管 IVYBM 受控 App。</t>
+          <t xml:space="preserve">默认填写“IVYBM 受控 App”；只有合同或 IVYBM 书面操作单明确要求时才填写“客户自持 App”。</t>
         </is>
       </c>
       <c r="G20" s="9" t="inlineStr">
@@ -2245,17 +2245,17 @@
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">M-17</t>
+          <t xml:space="preserve">M-15</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Webhook</t>
+          <t xml:space="preserve">Meta App</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">production 受控回调域名确认</t>
+          <t xml:space="preserve">客户自持 Meta App 名称</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
@@ -2265,12 +2265,12 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">必填</t>
+          <t xml:space="preserve">条件必填</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">系统回调路径固定为 /api/webhooks/meta；一期没有常驻 staging。</t>
+          <t xml:space="preserve">仅在 M-14 选择“客户自持 App”时填写；默认 IVYBM 受控 App 路径填“不适用”。</t>
         </is>
       </c>
       <c r="G21" s="9" t="inlineStr">
@@ -2287,17 +2287,17 @@
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">M-18</t>
+          <t xml:space="preserve">M-16</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Webhook</t>
+          <t xml:space="preserve">Meta App</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">META_WEBHOOK_ALLOWED_ACCOUNT_IDS allowlist 部署确认</t>
+          <t xml:space="preserve">客户自持 Meta App 最终管理员姓名 / 企业邮箱</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
@@ -2307,12 +2307,12 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">必填</t>
+          <t xml:space="preserve">条件必填</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">枚举：待确认,已确认部署,无需部署,被阻塞；只填状态，不填真实 ID 列表。</t>
+          <t xml:space="preserve">仅客户自持 App 时填写；不得要求客户登录或接管 IVYBM 受控 App。</t>
         </is>
       </c>
       <c r="G22" s="9" t="inlineStr">
@@ -2322,14 +2322,14 @@
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">待确认</t>
+          <t xml:space="preserve">未开始</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">M-19</t>
+          <t xml:space="preserve">M-17</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
@@ -2339,7 +2339,7 @@
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">META_WEBHOOK_APP_SECRET 部署确认</t>
+          <t xml:space="preserve">production 受控回调域名确认</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
@@ -2354,7 +2354,7 @@
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">枚举：待确认,已确认部署,无需部署,被阻塞；确认 App Secret 已写入服务器受控 storage，绝不写本表。</t>
+          <t xml:space="preserve">系统回调路径固定为 /api/webhooks/meta；一期没有常驻 staging。</t>
         </is>
       </c>
       <c r="G23" s="9" t="inlineStr">
@@ -2364,14 +2364,14 @@
       </c>
       <c r="H23" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">待确认</t>
+          <t xml:space="preserve">未开始</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">M-20</t>
+          <t xml:space="preserve">M-18</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">META_WEBHOOK_VERIFY_TOKEN 部署确认</t>
+          <t xml:space="preserve">META_WEBHOOK_ALLOWED_ACCOUNT_IDS allowlist 部署确认</t>
         </is>
       </c>
       <c r="D24" s="10" t="inlineStr">
@@ -2396,7 +2396,7 @@
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">枚举：待确认,已确认部署,无需部署,被阻塞；确认 Verify Token 已写入服务器受控 storage，绝不写本表。</t>
+          <t xml:space="preserve">枚举：待确认,已确认部署,无需部署,被阻塞；只填状态，不填真实 ID 列表。</t>
         </is>
       </c>
       <c r="G24" s="9" t="inlineStr">
@@ -2413,17 +2413,17 @@
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">M-21</t>
+          <t xml:space="preserve">M-19</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">联调</t>
+          <t xml:space="preserve">Webhook</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">测试发送方 Facebook / Instagram 账号负责人</t>
+          <t xml:space="preserve">META_WEBHOOK_APP_SECRET 部署确认</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">用于 Development Mode 联调。</t>
+          <t xml:space="preserve">枚举：待确认,已确认部署,无需部署,被阻塞；确认 App Secret 已写入服务器受控 storage，绝不写本表。</t>
         </is>
       </c>
       <c r="G25" s="9" t="inlineStr">
@@ -2448,24 +2448,24 @@
       </c>
       <c r="H25" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">未开始</t>
+          <t xml:space="preserve">待确认</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">M-22</t>
+          <t xml:space="preserve">M-20</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">审核</t>
+          <t xml:space="preserve">Webhook</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">是否同意提交 App Review 和录制演示</t>
+          <t xml:space="preserve">META_WEBHOOK_VERIFY_TOKEN 部署确认</t>
         </is>
       </c>
       <c r="D26" s="10" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">生产权限通常需要企业验证、说明与录屏。</t>
+          <t xml:space="preserve">枚举：待确认,已确认部署,无需部署,被阻塞；确认 Verify Token 已写入服务器受控 storage，绝不写本表。</t>
         </is>
       </c>
       <c r="G26" s="9" t="inlineStr">
@@ -2490,69 +2490,153 @@
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">未开始</t>
+          <t xml:space="preserve">待确认</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
+          <t xml:space="preserve">M-21</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">联调</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">测试发送方 Facebook / Instagram 账号负责人</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">必填</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">用于 Development Mode 联调。</t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H27" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未开始</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M-22</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">审核</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">是否同意提交 App Review 和录制演示</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">必填</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">生产权限通常需要企业验证、说明与录屏。</t>
+        </is>
+      </c>
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H28" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">未开始</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
           <t xml:space="preserve">M-23</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">发布</t>
         </is>
       </c>
-      <c r="C27" s="9" t="inlineStr">
+      <c r="C29" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Facebook / Instagram 图文发布受控测试意向</t>
         </is>
       </c>
-      <c r="D27" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E27" s="7" t="inlineStr">
+      <c r="D29" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">建议</t>
         </is>
       </c>
-      <c r="F27" s="9" t="inlineStr">
+      <c r="F29" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">不改变一期冻结范围；发布仍以 PublishJobs / PublishLogs / adapter 评审为前置条件，未评审通过不承诺自动联调。</t>
         </is>
       </c>
-      <c r="G27" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
-        </is>
-      </c>
-      <c r="H27" s="11" t="inlineStr">
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">通过受控方式提供；不要填密码、验证码、App Secret、Client Secret、OAuth Token 或银行卡信息。</t>
+        </is>
+      </c>
+      <c r="H29" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">未开始</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H27"/>
+  <autoFilter ref="A4:H29"/>
   <mergeCells count="2">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
   <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H10 H13 H14 H18 H19 H20 H21 H25 H26 H27">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H5 H6 H7 H8 H10 H11 H14 H15 H18 H20 H21 H22 H23 H27 H28 H29">
       <formula1>"未开始,已提供,待补充,不适用"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H9 H15">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H9 H16">
       <formula1>"未开始,待处理,已连接,已过期,被阻塞,已停用"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H11 H12 H16 H17">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H12 H13 H17 H19">
       <formula1>"未开始,待审核,已通过,被阻塞"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H22 H23 H24">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H24 H25 H26">
       <formula1>"待确认,已确认部署,无需部署,被阻塞"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2767,7 +2851,7 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">企业主页 URL 或希望创建的英文名</t>
+          <t xml:space="preserve">企业主页 URL 或客户拟用英文名</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
@@ -2782,7 +2866,7 @@
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">账号类型 = linkedin-organization；新建 Page 需品牌、官网、Logo、简介。</t>
+          <t xml:space="preserve">账号类型 = linkedin-organization；无主页由客户创建并保留 Super Admin，新建 Page 需品牌、官网、Logo、简介。</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
@@ -2824,7 +2908,7 @@
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">创建后补填；只填公开组织 ID。</t>
+          <t xml:space="preserve">客户创建/取得后补填；只填公开组织 ID。</t>
         </is>
       </c>
       <c r="G9" s="9" t="inlineStr">
@@ -3234,7 +3318,7 @@
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">TikTok Business Account 是否已有 / 需新建</t>
+          <t xml:space="preserve">TikTok Business Account 是否已有 / 需由客户新建</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
@@ -3249,7 +3333,7 @@
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">账号类型 = tiktok-business；提供链接或填写“需新建”。</t>
+          <t xml:space="preserve">账号类型 = tiktok-business；提供链接；无账号由客户自行注册/转换并保留 Owner。</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
@@ -3291,7 +3375,7 @@
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">创建后补填；只填公开账号 ID。</t>
+          <t xml:space="preserve">客户创建/取得后补填；只填公开账号 ID。</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
@@ -3486,7 +3570,7 @@
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">TikTok for Developers 账号是否已有 / 需新建</t>
+          <t xml:space="preserve">TikTok for Developers 账号是否已有 / 需由客户新建</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
@@ -3501,7 +3585,7 @@
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">仅在 TikTok-3 私信资格决策门已有“可申请”或“已批准”证据后填写；技术团队可协助，客户保留最终管理员。</t>
+          <t xml:space="preserve">仅在 TikTok-3 私信资格决策门已有“可申请”或“已批准”证据后填写；客户 Owner 自行创建并保留最终管理员。IVYBM 仅在书面授权后协助 App/API/Webhook 配置，不代注册。</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
@@ -4121,7 +4205,7 @@
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">客户最终接收企业邮箱、2FA、管理员权限的人</t>
+          <t xml:space="preserve">客户最终持有企业邮箱、2FA、管理员权限与恢复方式的负责人</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
@@ -4136,7 +4220,7 @@
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">账号开通后由其改密并保留恢复方式。</t>
+          <t xml:space="preserve">客户自行创建/持有账号后，由其保留恢复方式；IVYBM 不代注册、养号或恢复账号。</t>
         </is>
       </c>
       <c r="G13" s="9" t="inlineStr">

</xml_diff>